<commit_message>
Merge Suggestion cells across each record's full row span
Screenshot showed the new Suggestion columns leaving a bare, unmerged
single-height cell for records whose Failure Mode spans 2 Excel rows
(e.g. rows 18-19, merged in every other column for that record) - this
looked visually broken next to the rest of the merged row.

Data cells are now merged across min(source_excel_rows) to
max(source_excel_rows) for each of the 6 Suggestion columns, matching
however many rows that record actually spans in the original sheet
(1 row for the two torque entries, 2 rows for the others). Styling
(border/alignment/font) is copied from a real neighboring data cell
instead of using default/bare formatting, so it reads as part of the
same row instead of a bolted-on afterthought.

Removed find_data_row_for_excel_row(), now dead code since row spans are
read directly from source_excel_rows instead of inferred from an
existing column's merge range.
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -2470,20 +2470,20 @@
       <c r="AJ18" s="45" t="n"/>
       <c r="AK18" s="45" t="n"/>
       <c r="AL18" s="35" t="n"/>
-      <c r="AM18" t="n">
+      <c r="AM18" s="169" t="n">
         <v>8</v>
       </c>
-      <c r="AN18" t="inlineStr">
+      <c r="AN18" s="169" t="inlineStr">
         <is>
           <t>The End User effects list functional outcomes (no light or dim light) without any explicit safety or regulatory language; given the merged "scratch/damage" mode, the DAMAGE sub-mode can directly cause either total loss or degradation of the headlamp’s primary function, so the worst-case applicable definition is loss of primary function (8).</t>
         </is>
       </c>
-      <c r="AQ18" t="inlineStr">
+      <c r="AQ18" s="169" t="inlineStr">
         <is>
           <t>Add a mandatory barcode scan at the sequencing trolley that interlocks the station and blocks tool enable if the scanned headlamp PN/variant does not match the vehicle build sheet, preventing wrong-part selection/mix-up.</t>
         </is>
       </c>
-      <c r="AR18" t="inlineStr">
+      <c r="AR18" s="169" t="inlineStr">
         <is>
           <t>Merged failure mode: 1. Scratch on head lamp; 2. Damage on head lamp. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it reads like the cause for installing the wrong headlamp variant rather than for scratching/damaging the part. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
@@ -2577,20 +2577,20 @@
       <c r="AJ20" s="45" t="n"/>
       <c r="AK20" s="45" t="n"/>
       <c r="AL20" s="35" t="n"/>
-      <c r="AM20" t="n">
+      <c r="AM20" s="169" t="n">
         <v>8</v>
       </c>
-      <c r="AN20" t="inlineStr">
+      <c r="AN20" s="169" t="inlineStr">
         <is>
           <t>The End User effects list either a total loss of the headlamp function ('does not turn ON') or a degraded primary function ('dim light'), both directly plausible from wrong-part selection/mix-up; no safety or regulatory wording is stated. Per the table, these correspond to S=8 or S=7 respectively, with the row-level score set to the higher (8) due to merged/ambiguous mode effects.</t>
         </is>
       </c>
-      <c r="AQ20" t="inlineStr">
+      <c r="AQ20" s="169" t="inlineStr">
         <is>
           <t>Add a scan-and-verify lockout at the pick/scan step so the headlamp barcode must match the vehicle’s model code and the line prevents installation if a wrong part is scanned.</t>
         </is>
       </c>
-      <c r="AR20" t="inlineStr">
+      <c r="AR20" s="169" t="inlineStr">
         <is>
           <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2698,20 +2698,20 @@
       <c r="AJ22" s="45" t="n"/>
       <c r="AK22" s="45" t="n"/>
       <c r="AL22" s="35" t="n"/>
-      <c r="AM22" t="n">
+      <c r="AM22" s="169" t="n">
         <v>10</v>
       </c>
-      <c r="AN22" t="inlineStr">
+      <c r="AN22" s="169" t="inlineStr">
         <is>
           <t>The End User effect list explicitly states 'Increased risk of accident', which is a plausible consequence of the headlamp not turning on or reduced visibility caused by improper/poor connector locking. Per the table, this affects safe operation of the vehicle, so Severity is 10.</t>
         </is>
       </c>
-      <c r="AQ22" t="inlineStr">
+      <c r="AQ22" s="169" t="inlineStr">
         <is>
           <t>Add a poka‑yoke for the headlamp connectors: a latch‑engagement sensor or pull‑back test with line interlock that prevents process completion if the connector is not fully seated and locked.</t>
         </is>
       </c>
-      <c r="AR22" t="inlineStr">
+      <c r="AR22" s="169" t="inlineStr">
         <is>
           <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2829,20 +2829,20 @@
       <c r="AJ24" s="12" t="n"/>
       <c r="AK24" s="12" t="n"/>
       <c r="AL24" s="10" t="n"/>
-      <c r="AM24" t="n">
+      <c r="AM24" s="169" t="n">
         <v>10</v>
       </c>
-      <c r="AN24" t="inlineStr">
+      <c r="AN24" s="169" t="inlineStr">
         <is>
           <t>The End User effect explicitly states 'Increased risk of accident,' which is a direct and plausible consequence of a headlamp installed without required prefit bolts causing misalignment or compromised illumination. Per the Severity table, this affects safe operation of the vehicle, warranting a 10.</t>
         </is>
       </c>
-      <c r="AQ24" t="inlineStr">
+      <c r="AQ24" s="169" t="inlineStr">
         <is>
           <t>Install a DC torque tool with bolt-count and torque OK interlock that prevents station completion unless all headlamp bolts are started and torqued to 6 Nm per the SOS.</t>
         </is>
       </c>
-      <c r="AR24" t="inlineStr">
+      <c r="AR24" s="169" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2956,20 +2956,20 @@
       <c r="AJ26" s="12" t="n"/>
       <c r="AK26" s="12" t="n"/>
       <c r="AL26" s="10" t="n"/>
-      <c r="AM26" t="n">
+      <c r="AM26" s="169" t="n">
         <v>4</v>
       </c>
-      <c r="AN26" t="inlineStr">
+      <c r="AN26" s="169" t="inlineStr">
         <is>
           <t>Among the listed End User effects, the only direct outcome of 'failed to fit screws/not maintained gap' is 'rattling or vibration noise during driving', which falls under very objectionable sound/vibration. The more severe-sounding effects (lens crack, bulb burnout, water ingress) require additional unstated failures and are therefore indirect for this mode/cause.</t>
         </is>
       </c>
-      <c r="AQ26" t="inlineStr">
+      <c r="AQ26" s="169" t="inlineStr">
         <is>
           <t>Add an in-station fixture with hard locators and an interlocked gap/fastener verification (camera or go/no-go gauge plus screw-counting torque tool) that blocks OK-to-ship unless uniform gaps are met and all screws are installed/torqued.</t>
         </is>
       </c>
-      <c r="AR26" t="inlineStr">
+      <c r="AR26" s="169" t="inlineStr">
         <is>
           <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap. Cause/Mode mismatch: The stated Cause addresses only non-uniform gaps to the fender; it does not explain the 'failed to fit screws' portion of the Failure Mode.</t>
         </is>
@@ -3090,20 +3090,20 @@
       <c r="AJ28" s="12" t="n"/>
       <c r="AK28" s="12" t="n"/>
       <c r="AL28" s="10" t="n"/>
-      <c r="AM28" t="n">
+      <c r="AM28" s="169" t="n">
         <v>4</v>
       </c>
-      <c r="AN28" t="inlineStr">
+      <c r="AN28" s="169" t="inlineStr">
         <is>
           <t>The direct customer-facing outcome of an under-torqued headlamp mount is rattle/vibration noise while driving, which fits the table’s NVH category. This is reasonably treated as very objectionable NVH, aligning with Severity 4.</t>
         </is>
       </c>
-      <c r="AQ28" t="inlineStr">
+      <c r="AQ28" s="169" t="inlineStr">
         <is>
           <t>Install a torque-controlled, calibrated electric driver programmed to 6 Nm with OK/NOK lockout to prevent under-torque from operator mistake, wrong tool use, or miscalibration.</t>
         </is>
       </c>
-      <c r="AR28" t="inlineStr">
+      <c r="AR28" s="169" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3148,20 +3148,20 @@
       <c r="AJ29" s="12" t="n"/>
       <c r="AK29" s="12" t="n"/>
       <c r="AL29" s="10" t="n"/>
-      <c r="AM29" t="n">
+      <c r="AM29" s="169" t="n">
         <v>4</v>
       </c>
-      <c r="AN29" t="inlineStr">
+      <c r="AN29" s="169" t="inlineStr">
         <is>
           <t>The direct customer outcomes of this torque error are a cracked/broken lens (over‑torque) or rattling/vibration noise (under‑torque), which are NVH/appearance issues; there is no explicit accident/injury or regulatory noncompliance stated, and loss/degradation of illumination is not directly attributed to this torque error in the listed effects.</t>
         </is>
       </c>
-      <c r="AQ29" t="inlineStr">
+      <c r="AQ29" s="169" t="inlineStr">
         <is>
           <t>Install a DC torque tool programmed to 6 Nm with barcode-linked job selection and OK/NOK lockout so the station cannot proceed if the specified torque is not achieved, preventing wrong tool use and calibration drift from producing under/over‑torque.</t>
         </is>
       </c>
-      <c r="AR29" t="inlineStr">
+      <c r="AR29" s="169" t="inlineStr">
         <is>
           <t>Merged failure mode: 1. Under‑torque (torque not achieved); 2. Over‑torque. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3169,7 +3169,7 @@
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="132">
+  <mergeCells count="152">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
@@ -3186,6 +3186,7 @@
     <mergeCell ref="D12:F12"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G13:L14"/>
+    <mergeCell ref="AR24:AR25"/>
     <mergeCell ref="K9:T9"/>
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
@@ -3193,11 +3194,14 @@
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
     <mergeCell ref="V15:V17"/>
     <mergeCell ref="Y18:Y21"/>
     <mergeCell ref="R18:S18"/>
+    <mergeCell ref="AM18:AM19"/>
     <mergeCell ref="T27:U27"/>
+    <mergeCell ref="AR18:AR19"/>
     <mergeCell ref="AP15:AP17"/>
     <mergeCell ref="K8:T8"/>
     <mergeCell ref="AR15:AR17"/>
@@ -3205,19 +3209,26 @@
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="M22:N25"/>
     <mergeCell ref="T24:U24"/>
+    <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
+    <mergeCell ref="AN24:AN25"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="AN20:AN21"/>
+    <mergeCell ref="AQ22:AQ23"/>
+    <mergeCell ref="AN26:AN27"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="R25:S25"/>
     <mergeCell ref="Z18:Z21"/>
     <mergeCell ref="T25:U25"/>
+    <mergeCell ref="AN22:AN23"/>
     <mergeCell ref="P18:Q19"/>
     <mergeCell ref="AQ15:AQ17"/>
     <mergeCell ref="Y23:Y25"/>
     <mergeCell ref="Z27:Z29"/>
+    <mergeCell ref="AR20:AR21"/>
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="M15:N17"/>
     <mergeCell ref="G18:H29"/>
@@ -3233,6 +3244,7 @@
     <mergeCell ref="AC15:AC17"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
+    <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AD15:AD17"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="A7:C7"/>
@@ -3241,6 +3253,7 @@
     <mergeCell ref="A13:F14"/>
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
+    <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="P15:Q17"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="AH15:AH17"/>
@@ -3249,20 +3262,24 @@
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="O18:O21"/>
     <mergeCell ref="M18:N21"/>
+    <mergeCell ref="AN18:AN19"/>
     <mergeCell ref="A1:R2"/>
     <mergeCell ref="AL15:AL17"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="R27:S27"/>
     <mergeCell ref="R20:S20"/>
+    <mergeCell ref="AM20:AM21"/>
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="P22:Q23"/>
+    <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
     <mergeCell ref="T19:U19"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
+    <mergeCell ref="AM26:AM27"/>
     <mergeCell ref="A3:H4"/>
     <mergeCell ref="P29:Q29"/>
     <mergeCell ref="I15:J17"/>
@@ -3281,11 +3298,13 @@
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="R24:S24"/>
+    <mergeCell ref="AM24:AM25"/>
     <mergeCell ref="M13:S14"/>
     <mergeCell ref="P24:Q25"/>
     <mergeCell ref="AM13:AR14"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="Z15:Z17"/>
+    <mergeCell ref="AQ18:AQ19"/>
     <mergeCell ref="AB15:AB17"/>
     <mergeCell ref="R21:S21"/>
     <mergeCell ref="T21:U21"/>
@@ -3300,6 +3319,7 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>
   </mergeCells>

</xml_diff>

<commit_message>
Remove fill from top Suggestion header, widen new columns for readability
Two issues from the plant's screenshot: the purple fill was applied to
the whole merged "Suggestion" top header, when only the sub-column
headers below it (Severity, Occurrence, Detection, Prevention, etc.)
should carry the distinct color - matching how the sheet's own sibling
sections (e.g. "Optimization (Step6)") leave their top-level header
unfilled. Also, wrapped text in the new text-heavy columns (Severity
Note, Detection, Prevention, Remark) was unreadable at the sheet's
default column width.

Fixed: section_cell now copies style without a fill override (plain,
like its siblings); sub-column headers keep the purple fill. Added
explicit column widths - narrow for Severity/Occurrence, wider for the
text-heavy columns (Remark widest at 55, since it can carry several
concatenated flags).
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -1216,7 +1216,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1607,6 +1607,12 @@
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
     <col width="12.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="39" max="39"/>
+    <col width="32" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="32" customWidth="1" min="42" max="42"/>
+    <col width="38" customWidth="1" min="43" max="43"/>
+    <col width="55" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">

</xml_diff>